<commit_message>
Add confirmed Poomsae question
</commit_message>
<xml_diff>
--- a/content/production/questions.xlsx
+++ b/content/production/questions.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5354" uniqueCount="3029">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5362" uniqueCount="3034">
   <si>
     <t>category</t>
   </si>
@@ -8852,6 +8852,21 @@
   </si>
   <si>
     <t>Άτομα με αναπηρικά καροτσάκια</t>
+  </si>
+  <si>
+    <t>Η αγωνιστική περιοχή στο Poomsae είναι:</t>
+  </si>
+  <si>
+    <t>12x12</t>
+  </si>
+  <si>
+    <t>10x10</t>
+  </si>
+  <si>
+    <t>8x8</t>
+  </si>
+  <si>
+    <t>Δεν υπάρχει οριοθέτηση</t>
   </si>
   <si>
     <t>Στον έλεγχο των αθλητών ο διαιτητής ελέγχει αν:</t>
@@ -9491,7 +9506,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:N667"/>
+  <dimension ref="A1:N668"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="28" customWidth="1"/>
@@ -31620,7 +31635,7 @@
         <v>2950</v>
       </c>
       <c r="F650" s="2" t="s">
-        <v>1405</v>
+        <v>2951</v>
       </c>
       <c r="G650" s="2"/>
       <c r="H650" s="2"/>
@@ -31634,7 +31649,7 @@
         <v>2931</v>
       </c>
       <c r="N650" s="2">
-        <v>36</v>
+        <v>31</v>
       </c>
     </row>
     <row r="651" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -31642,22 +31657,24 @@
         <v>2924</v>
       </c>
       <c r="B651" s="2" t="s">
-        <v>2951</v>
+        <v>2952</v>
       </c>
       <c r="C651" s="2" t="s">
-        <v>2952</v>
+        <v>2953</v>
       </c>
       <c r="D651" s="2" t="s">
-        <v>2953</v>
+        <v>2954</v>
       </c>
       <c r="E651" s="2" t="s">
-        <v>2954</v>
-      </c>
-      <c r="F651" s="2"/>
+        <v>2955</v>
+      </c>
+      <c r="F651" s="2" t="s">
+        <v>1405</v>
+      </c>
       <c r="G651" s="2"/>
       <c r="H651" s="2"/>
       <c r="I651" s="2" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="J651" s="2"/>
       <c r="K651" s="2"/>
@@ -31666,7 +31683,7 @@
         <v>2931</v>
       </c>
       <c r="N651" s="2">
-        <v>42</v>
+        <v>36</v>
       </c>
     </row>
     <row r="652" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -31674,26 +31691,22 @@
         <v>2924</v>
       </c>
       <c r="B652" s="2" t="s">
-        <v>2955</v>
+        <v>2956</v>
       </c>
       <c r="C652" s="2" t="s">
-        <v>2956</v>
+        <v>2957</v>
       </c>
       <c r="D652" s="2" t="s">
-        <v>2957</v>
+        <v>2958</v>
       </c>
       <c r="E652" s="2" t="s">
-        <v>2958</v>
-      </c>
-      <c r="F652" s="2" t="s">
         <v>2959</v>
       </c>
-      <c r="G652" s="2" t="s">
-        <v>1405</v>
-      </c>
+      <c r="F652" s="2"/>
+      <c r="G652" s="2"/>
       <c r="H652" s="2"/>
       <c r="I652" s="2" t="s">
-        <v>2930</v>
+        <v>49</v>
       </c>
       <c r="J652" s="2"/>
       <c r="K652" s="2"/>
@@ -31702,7 +31715,7 @@
         <v>2931</v>
       </c>
       <c r="N652" s="2">
-        <v>56</v>
+        <v>42</v>
       </c>
     </row>
     <row r="653" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -31724,10 +31737,12 @@
       <c r="F653" s="2" t="s">
         <v>2964</v>
       </c>
-      <c r="G653" s="2"/>
+      <c r="G653" s="2" t="s">
+        <v>1405</v>
+      </c>
       <c r="H653" s="2"/>
       <c r="I653" s="2" t="s">
-        <v>20</v>
+        <v>2930</v>
       </c>
       <c r="J653" s="2"/>
       <c r="K653" s="2"/>
@@ -31736,7 +31751,7 @@
         <v>2931</v>
       </c>
       <c r="N653" s="2">
-        <v>63</v>
+        <v>56</v>
       </c>
     </row>
     <row r="654" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -31756,12 +31771,12 @@
         <v>2968</v>
       </c>
       <c r="F654" s="2" t="s">
-        <v>1405</v>
+        <v>2969</v>
       </c>
       <c r="G654" s="2"/>
       <c r="H654" s="2"/>
       <c r="I654" s="2" t="s">
-        <v>27</v>
+        <v>20</v>
       </c>
       <c r="J654" s="2"/>
       <c r="K654" s="2"/>
@@ -31770,7 +31785,7 @@
         <v>2931</v>
       </c>
       <c r="N654" s="2">
-        <v>69</v>
+        <v>63</v>
       </c>
     </row>
     <row r="655" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -31778,19 +31793,19 @@
         <v>2924</v>
       </c>
       <c r="B655" s="2" t="s">
-        <v>2969</v>
+        <v>2970</v>
       </c>
       <c r="C655" s="2" t="s">
-        <v>2970</v>
+        <v>2971</v>
       </c>
       <c r="D655" s="2" t="s">
-        <v>2971</v>
+        <v>2972</v>
       </c>
       <c r="E655" s="2" t="s">
-        <v>2972</v>
+        <v>2973</v>
       </c>
       <c r="F655" s="2" t="s">
-        <v>1477</v>
+        <v>1405</v>
       </c>
       <c r="G655" s="2"/>
       <c r="H655" s="2"/>
@@ -31804,7 +31819,7 @@
         <v>2931</v>
       </c>
       <c r="N655" s="2">
-        <v>75</v>
+        <v>69</v>
       </c>
     </row>
     <row r="656" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -31812,24 +31827,24 @@
         <v>2924</v>
       </c>
       <c r="B656" s="2" t="s">
-        <v>2973</v>
+        <v>2974</v>
       </c>
       <c r="C656" s="2" t="s">
-        <v>2974</v>
+        <v>2975</v>
       </c>
       <c r="D656" s="2" t="s">
-        <v>2975</v>
+        <v>2976</v>
       </c>
       <c r="E656" s="2" t="s">
-        <v>2976</v>
+        <v>2977</v>
       </c>
       <c r="F656" s="2" t="s">
-        <v>2977</v>
+        <v>1477</v>
       </c>
       <c r="G656" s="2"/>
       <c r="H656" s="2"/>
       <c r="I656" s="2" t="s">
-        <v>20</v>
+        <v>27</v>
       </c>
       <c r="J656" s="2"/>
       <c r="K656" s="2"/>
@@ -31838,7 +31853,7 @@
         <v>2931</v>
       </c>
       <c r="N656" s="2">
-        <v>82</v>
+        <v>75</v>
       </c>
     </row>
     <row r="657" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -31858,12 +31873,12 @@
         <v>2981</v>
       </c>
       <c r="F657" s="2" t="s">
-        <v>1477</v>
+        <v>2982</v>
       </c>
       <c r="G657" s="2"/>
       <c r="H657" s="2"/>
       <c r="I657" s="2" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="J657" s="2"/>
       <c r="K657" s="2"/>
@@ -31872,7 +31887,7 @@
         <v>2931</v>
       </c>
       <c r="N657" s="2">
-        <v>89</v>
+        <v>82</v>
       </c>
     </row>
     <row r="658" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -31880,24 +31895,24 @@
         <v>2924</v>
       </c>
       <c r="B658" s="2" t="s">
-        <v>2982</v>
+        <v>2983</v>
       </c>
       <c r="C658" s="2" t="s">
-        <v>2983</v>
+        <v>2984</v>
       </c>
       <c r="D658" s="2" t="s">
-        <v>2984</v>
+        <v>2985</v>
       </c>
       <c r="E658" s="2" t="s">
-        <v>2985</v>
+        <v>2986</v>
       </c>
       <c r="F658" s="2" t="s">
-        <v>2986</v>
+        <v>1477</v>
       </c>
       <c r="G658" s="2"/>
       <c r="H658" s="2"/>
       <c r="I658" s="2" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="J658" s="2"/>
       <c r="K658" s="2"/>
@@ -31906,7 +31921,7 @@
         <v>2931</v>
       </c>
       <c r="N658" s="2">
-        <v>95</v>
+        <v>89</v>
       </c>
     </row>
     <row r="659" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -31940,7 +31955,7 @@
         <v>2931</v>
       </c>
       <c r="N659" s="2">
-        <v>101</v>
+        <v>95</v>
       </c>
     </row>
     <row r="660" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -31960,14 +31975,12 @@
         <v>2995</v>
       </c>
       <c r="F660" s="2" t="s">
-        <v>1477</v>
-      </c>
-      <c r="G660" s="2" t="s">
-        <v>1405</v>
-      </c>
+        <v>2996</v>
+      </c>
+      <c r="G660" s="2"/>
       <c r="H660" s="2"/>
       <c r="I660" s="2" t="s">
-        <v>2930</v>
+        <v>27</v>
       </c>
       <c r="J660" s="2"/>
       <c r="K660" s="2"/>
@@ -31976,7 +31989,7 @@
         <v>2931</v>
       </c>
       <c r="N660" s="2">
-        <v>107</v>
+        <v>101</v>
       </c>
     </row>
     <row r="661" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -31984,24 +31997,26 @@
         <v>2924</v>
       </c>
       <c r="B661" s="2" t="s">
-        <v>2996</v>
+        <v>2997</v>
       </c>
       <c r="C661" s="2" t="s">
-        <v>2997</v>
+        <v>2998</v>
       </c>
       <c r="D661" s="2" t="s">
-        <v>2998</v>
+        <v>2999</v>
       </c>
       <c r="E661" s="2" t="s">
-        <v>2999</v>
+        <v>3000</v>
       </c>
       <c r="F661" s="2" t="s">
-        <v>3000</v>
-      </c>
-      <c r="G661" s="2"/>
+        <v>1477</v>
+      </c>
+      <c r="G661" s="2" t="s">
+        <v>1405</v>
+      </c>
       <c r="H661" s="2"/>
       <c r="I661" s="2" t="s">
-        <v>27</v>
+        <v>2930</v>
       </c>
       <c r="J661" s="2"/>
       <c r="K661" s="2"/>
@@ -32010,7 +32025,7 @@
         <v>2931</v>
       </c>
       <c r="N661" s="2">
-        <v>114</v>
+        <v>107</v>
       </c>
     </row>
     <row r="662" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -32030,12 +32045,12 @@
         <v>3004</v>
       </c>
       <c r="F662" s="2" t="s">
-        <v>1477</v>
+        <v>3005</v>
       </c>
       <c r="G662" s="2"/>
       <c r="H662" s="2"/>
       <c r="I662" s="2" t="s">
-        <v>38</v>
+        <v>27</v>
       </c>
       <c r="J662" s="2"/>
       <c r="K662" s="2"/>
@@ -32044,7 +32059,7 @@
         <v>2931</v>
       </c>
       <c r="N662" s="2">
-        <v>122</v>
+        <v>114</v>
       </c>
     </row>
     <row r="663" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -32052,19 +32067,19 @@
         <v>2924</v>
       </c>
       <c r="B663" s="2" t="s">
-        <v>3005</v>
+        <v>3006</v>
       </c>
       <c r="C663" s="2" t="s">
-        <v>3006</v>
+        <v>3007</v>
       </c>
       <c r="D663" s="2" t="s">
-        <v>3007</v>
+        <v>3008</v>
       </c>
       <c r="E663" s="2" t="s">
-        <v>3008</v>
+        <v>3009</v>
       </c>
       <c r="F663" s="2" t="s">
-        <v>3009</v>
+        <v>1477</v>
       </c>
       <c r="G663" s="2"/>
       <c r="H663" s="2"/>
@@ -32078,7 +32093,7 @@
         <v>2931</v>
       </c>
       <c r="N663" s="2">
-        <v>128</v>
+        <v>122</v>
       </c>
     </row>
     <row r="664" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -32103,7 +32118,7 @@
       <c r="G664" s="2"/>
       <c r="H664" s="2"/>
       <c r="I664" s="2" t="s">
-        <v>20</v>
+        <v>38</v>
       </c>
       <c r="J664" s="2"/>
       <c r="K664" s="2"/>
@@ -32112,7 +32127,7 @@
         <v>2931</v>
       </c>
       <c r="N664" s="2">
-        <v>134</v>
+        <v>128</v>
       </c>
     </row>
     <row r="665" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -32146,7 +32161,7 @@
         <v>2931</v>
       </c>
       <c r="N665" s="2">
-        <v>140</v>
+        <v>134</v>
       </c>
     </row>
     <row r="666" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -32171,7 +32186,7 @@
       <c r="G666" s="2"/>
       <c r="H666" s="2"/>
       <c r="I666" s="2" t="s">
-        <v>38</v>
+        <v>20</v>
       </c>
       <c r="J666" s="2"/>
       <c r="K666" s="2"/>
@@ -32180,7 +32195,7 @@
         <v>2931</v>
       </c>
       <c r="N666" s="2">
-        <v>146</v>
+        <v>140</v>
       </c>
     </row>
     <row r="667" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
@@ -32200,12 +32215,12 @@
         <v>3028</v>
       </c>
       <c r="F667" s="2" t="s">
-        <v>1477</v>
+        <v>3029</v>
       </c>
       <c r="G667" s="2"/>
       <c r="H667" s="2"/>
       <c r="I667" s="2" t="s">
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="J667" s="2"/>
       <c r="K667" s="2"/>
@@ -32214,11 +32229,45 @@
         <v>2931</v>
       </c>
       <c r="N667" s="2">
+        <v>146</v>
+      </c>
+    </row>
+    <row r="668" spans="1:14" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A668" s="2" t="s">
+        <v>2924</v>
+      </c>
+      <c r="B668" s="2" t="s">
+        <v>3030</v>
+      </c>
+      <c r="C668" s="2" t="s">
+        <v>3031</v>
+      </c>
+      <c r="D668" s="2" t="s">
+        <v>3032</v>
+      </c>
+      <c r="E668" s="2" t="s">
+        <v>3033</v>
+      </c>
+      <c r="F668" s="2" t="s">
+        <v>1477</v>
+      </c>
+      <c r="G668" s="2"/>
+      <c r="H668" s="2"/>
+      <c r="I668" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J668" s="2"/>
+      <c r="K668" s="2"/>
+      <c r="L668" s="2"/>
+      <c r="M668" s="2" t="s">
+        <v>2931</v>
+      </c>
+      <c r="N668" s="2">
         <v>152</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:N667"/>
+  <autoFilter ref="A1:N668"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>
 </worksheet>

</xml_diff>